<commit_message>
auto: Çeyreklik bilanço verileri güncellendi [20.10.2026]
</commit_message>
<xml_diff>
--- a/Temel_Analiz_Omurga.xlsx
+++ b/Temel_Analiz_Omurga.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Tetik Bölgesi</t>
+          <t>Temel Skor</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
@@ -552,7 +552,9 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>47</v>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -604,7 +606,9 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="n">
+        <v>39</v>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -656,10 +660,12 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="n">
+        <v>30</v>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%46.4)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -712,7 +718,9 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>40</v>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -764,7 +772,9 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="P6" t="n">
+        <v>49</v>
+      </c>
       <c r="Q6" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -816,7 +826,9 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="n">
+        <v>57</v>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -868,7 +880,9 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="n">
+        <v>55</v>
+      </c>
       <c r="Q8" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -920,7 +934,9 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="n">
+        <v>34</v>
+      </c>
       <c r="Q9" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -972,7 +988,9 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="n">
+        <v>64</v>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1028,7 +1046,9 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="n">
+        <v>55</v>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -1080,7 +1100,9 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>49</v>
+      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1136,7 +1158,9 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="n">
+        <v>70</v>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -1192,7 +1216,9 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="n">
+        <v>100</v>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -1244,7 +1270,9 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="n">
+        <v>30</v>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1296,7 +1324,9 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>57</v>
+      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1348,7 +1378,9 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>77</v>
+      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1400,7 +1432,9 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>60</v>
+      </c>
       <c r="Q18" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1452,7 +1486,9 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>40</v>
+      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1504,7 +1540,9 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="n">
+        <v>57</v>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1556,10 +1594,12 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="n">
+        <v>13</v>
+      </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%24.4)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr"/>
@@ -1608,7 +1648,9 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
+      <c r="P22" t="n">
+        <v>56</v>
+      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1660,7 +1702,9 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="n">
+        <v>56</v>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1712,7 +1756,9 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>36</v>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1764,7 +1810,9 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>40</v>
+      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1816,7 +1864,9 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>71</v>
+      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1868,7 +1918,9 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>48</v>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -1920,10 +1972,12 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="n">
+        <v>25</v>
+      </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%5.1)</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
@@ -1972,10 +2026,12 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="n">
+        <v>34</v>
+      </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%17.9)</t>
         </is>
       </c>
       <c r="R29" t="inlineStr"/>
@@ -2024,10 +2080,12 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>22</v>
+      </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%17.5)</t>
         </is>
       </c>
       <c r="R30" t="inlineStr"/>
@@ -2076,10 +2134,12 @@
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>30</v>
+      </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%14.9)</t>
         </is>
       </c>
       <c r="R31" t="inlineStr"/>
@@ -2128,7 +2188,9 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>38</v>
+      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2180,7 +2242,9 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>31</v>
+      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2236,7 +2300,9 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
       <c r="Q34" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2288,7 +2354,9 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
+      <c r="P35" t="n">
+        <v>65</v>
+      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2340,7 +2408,9 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
+      <c r="P36" t="n">
+        <v>36</v>
+      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2392,7 +2462,9 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" t="n">
+        <v>55</v>
+      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2444,10 +2516,12 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
+      <c r="P38" t="n">
+        <v>14</v>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%13.7)</t>
         </is>
       </c>
       <c r="R38" t="inlineStr"/>
@@ -2496,7 +2570,9 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
+      <c r="P39" t="n">
+        <v>65</v>
+      </c>
       <c r="Q39" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2548,10 +2624,12 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
+      <c r="P40" t="n">
+        <v>23</v>
+      </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%5.9)</t>
         </is>
       </c>
       <c r="R40" t="inlineStr"/>
@@ -2600,7 +2678,9 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
+      <c r="P41" t="n">
+        <v>58</v>
+      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2652,7 +2732,9 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
+      <c r="P42" t="n">
+        <v>51</v>
+      </c>
       <c r="Q42" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2704,10 +2786,12 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
+      <c r="P43" t="n">
+        <v>18</v>
+      </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%50.3)</t>
         </is>
       </c>
       <c r="R43" t="inlineStr"/>
@@ -2756,7 +2840,9 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
+      <c r="P44" t="n">
+        <v>60</v>
+      </c>
       <c r="Q44" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2812,7 +2898,9 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
+      <c r="P45" t="n">
+        <v>70</v>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -2864,10 +2952,12 @@
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
+      <c r="P46" t="n">
+        <v>24</v>
+      </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%51.8)</t>
         </is>
       </c>
       <c r="R46" t="inlineStr"/>
@@ -2916,7 +3006,9 @@
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
+      <c r="P47" t="n">
+        <v>60</v>
+      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -2968,7 +3060,9 @@
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
+      <c r="P48" t="n">
+        <v>77</v>
+      </c>
       <c r="Q48" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3020,7 +3114,9 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
+      <c r="P49" t="n">
+        <v>73</v>
+      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3072,7 +3168,9 @@
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
+      <c r="P50" t="n">
+        <v>61</v>
+      </c>
       <c r="Q50" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3128,7 +3226,9 @@
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
+      <c r="P51" t="n">
+        <v>25</v>
+      </c>
       <c r="Q51" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -3180,7 +3280,9 @@
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
+      <c r="P52" t="n">
+        <v>23</v>
+      </c>
       <c r="Q52" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3236,7 +3338,9 @@
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
+      <c r="P53" t="n">
+        <v>40</v>
+      </c>
       <c r="Q53" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -3288,7 +3392,9 @@
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
+      <c r="P54" t="n">
+        <v>68</v>
+      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3344,7 +3450,9 @@
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
+      <c r="P55" t="n">
+        <v>70</v>
+      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -3396,7 +3504,9 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
+      <c r="P56" t="n">
+        <v>32</v>
+      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3448,7 +3558,9 @@
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
+      <c r="P57" t="n">
+        <v>43</v>
+      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3500,7 +3612,9 @@
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
+      <c r="P58" t="n">
+        <v>53</v>
+      </c>
       <c r="Q58" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3552,10 +3666,12 @@
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
+      <c r="P59" t="n">
+        <v>9</v>
+      </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%45.4)</t>
         </is>
       </c>
       <c r="R59" t="inlineStr"/>
@@ -3604,7 +3720,9 @@
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
+      <c r="P60" t="n">
+        <v>27</v>
+      </c>
       <c r="Q60" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3656,7 +3774,9 @@
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
+      <c r="P61" t="n">
+        <v>62</v>
+      </c>
       <c r="Q61" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3708,7 +3828,9 @@
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
+      <c r="P62" t="n">
+        <v>71</v>
+      </c>
       <c r="Q62" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3760,7 +3882,9 @@
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
+      <c r="P63" t="n">
+        <v>55</v>
+      </c>
       <c r="Q63" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3812,7 +3936,9 @@
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
+      <c r="P64" t="n">
+        <v>45</v>
+      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3864,10 +3990,12 @@
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
+      <c r="P65" t="n">
+        <v>34</v>
+      </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%16.2)</t>
         </is>
       </c>
       <c r="R65" t="inlineStr"/>
@@ -3916,7 +4044,9 @@
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
+      <c r="P66" t="n">
+        <v>46</v>
+      </c>
       <c r="Q66" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -3968,10 +4098,12 @@
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
+      <c r="P67" t="n">
+        <v>13</v>
+      </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%6.0)</t>
         </is>
       </c>
       <c r="R67" t="inlineStr"/>
@@ -4020,7 +4152,9 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
+      <c r="P68" t="n">
+        <v>11</v>
+      </c>
       <c r="Q68" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4072,7 +4206,9 @@
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
+      <c r="P69" t="n">
+        <v>61</v>
+      </c>
       <c r="Q69" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4124,10 +4260,12 @@
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
+      <c r="P70" t="n">
+        <v>24</v>
+      </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%95.7)</t>
         </is>
       </c>
       <c r="R70" t="inlineStr"/>
@@ -4176,7 +4314,9 @@
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
+      <c r="P71" t="n">
+        <v>34</v>
+      </c>
       <c r="Q71" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4228,7 +4368,9 @@
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
+      <c r="P72" t="n">
+        <v>14</v>
+      </c>
       <c r="Q72" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4280,7 +4422,9 @@
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
+      <c r="P73" t="n">
+        <v>63</v>
+      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4332,7 +4476,9 @@
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
+      <c r="P74" t="n">
+        <v>61</v>
+      </c>
       <c r="Q74" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4384,7 +4530,9 @@
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr"/>
+      <c r="P75" t="n">
+        <v>38</v>
+      </c>
       <c r="Q75" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4436,7 +4584,9 @@
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
+      <c r="P76" t="n">
+        <v>23</v>
+      </c>
       <c r="Q76" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4488,7 +4638,9 @@
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
+      <c r="P77" t="n">
+        <v>45</v>
+      </c>
       <c r="Q77" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4540,7 +4692,9 @@
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr"/>
+      <c r="P78" t="n">
+        <v>38</v>
+      </c>
       <c r="Q78" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4592,7 +4746,9 @@
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" t="inlineStr"/>
+      <c r="P79" t="n">
+        <v>33</v>
+      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4644,7 +4800,9 @@
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
+      <c r="P80" t="n">
+        <v>57</v>
+      </c>
       <c r="Q80" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4696,10 +4854,12 @@
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
+      <c r="P81" t="n">
+        <v>11</v>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%7.0)</t>
         </is>
       </c>
       <c r="R81" t="inlineStr"/>
@@ -4748,10 +4908,12 @@
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
+      <c r="P82" t="n">
+        <v>26</v>
+      </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%6.3)</t>
         </is>
       </c>
       <c r="R82" t="inlineStr"/>
@@ -4800,10 +4962,12 @@
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
+      <c r="P83" t="n">
+        <v>55</v>
+      </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%50.1)</t>
         </is>
       </c>
       <c r="R83" t="inlineStr"/>
@@ -4852,7 +5016,9 @@
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
+      <c r="P84" t="n">
+        <v>46</v>
+      </c>
       <c r="Q84" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4904,7 +5070,9 @@
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
+      <c r="P85" t="n">
+        <v>44</v>
+      </c>
       <c r="Q85" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -4956,10 +5124,12 @@
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" t="inlineStr"/>
+      <c r="P86" t="n">
+        <v>33</v>
+      </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>🚨 RİSKLİ (%24.0)</t>
         </is>
       </c>
       <c r="R86" t="inlineStr"/>
@@ -5008,7 +5178,9 @@
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
+      <c r="P87" t="n">
+        <v>59</v>
+      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5060,7 +5232,9 @@
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
+      <c r="P88" t="n">
+        <v>55</v>
+      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5112,7 +5286,9 @@
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
+      <c r="P89" t="n">
+        <v>57</v>
+      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5164,7 +5340,9 @@
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
+      <c r="P90" t="n">
+        <v>49</v>
+      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5220,7 +5398,9 @@
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" t="inlineStr"/>
+      <c r="P91" t="n">
+        <v>70</v>
+      </c>
       <c r="Q91" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -5272,10 +5452,12 @@
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr"/>
+      <c r="P92" t="n">
+        <v>19</v>
+      </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%9.0)</t>
         </is>
       </c>
       <c r="R92" t="inlineStr"/>
@@ -5324,7 +5506,9 @@
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" t="inlineStr"/>
+      <c r="P93" t="n">
+        <v>35</v>
+      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5376,7 +5560,9 @@
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" t="inlineStr"/>
+      <c r="P94" t="n">
+        <v>38</v>
+      </c>
       <c r="Q94" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5428,7 +5614,9 @@
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
+      <c r="P95" t="n">
+        <v>75</v>
+      </c>
       <c r="Q95" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5484,7 +5672,9 @@
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
+      <c r="P96" t="n">
+        <v>100</v>
+      </c>
       <c r="Q96" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -5536,7 +5726,9 @@
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
+      <c r="P97" t="n">
+        <v>51</v>
+      </c>
       <c r="Q97" t="inlineStr">
         <is>
           <t>✅ Temiz</t>
@@ -5592,7 +5784,9 @@
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
-      <c r="P98" t="inlineStr"/>
+      <c r="P98" t="n">
+        <v>40</v>
+      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -5644,10 +5838,12 @@
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
-      <c r="P99" t="inlineStr"/>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%6.1)</t>
         </is>
       </c>
       <c r="R99" t="inlineStr"/>
@@ -5700,7 +5896,9 @@
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" t="inlineStr"/>
+      <c r="P100" t="n">
+        <v>40</v>
+      </c>
       <c r="Q100" t="inlineStr">
         <is>
           <t>✅ Finans / Muaf</t>
@@ -5752,10 +5950,12 @@
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" t="inlineStr"/>
+      <c r="P101" t="n">
+        <v>4</v>
+      </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>✅ Temiz</t>
+          <t>⚠️ Dikkat (%10.6)</t>
         </is>
       </c>
       <c r="R101" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: Çeyreklik bilanço verileri güncellendi [26.10.2026]
</commit_message>
<xml_diff>
--- a/Temel_Analiz_Omurga.xlsx
+++ b/Temel_Analiz_Omurga.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -839,7 +839,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -893,7 +893,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1001,7 +1001,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1113,7 +1113,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1229,7 +1229,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1391,7 +1391,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1445,7 +1445,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1553,7 +1553,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1661,7 +1661,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1715,7 +1715,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1769,7 +1769,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1823,7 +1823,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1931,7 +1931,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1985,7 +1985,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2255,7 +2255,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2313,7 +2313,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2529,7 +2529,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2649,25 +2649,25 @@
         <v>7</v>
       </c>
       <c r="D41" t="n">
-        <v>4.38</v>
+        <v>4.34</v>
       </c>
       <c r="E41" t="n">
-        <v>0.014</v>
+        <v>0.0148</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0906</v>
+        <v>0.0987</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0263</v>
+        <v>0.0275</v>
       </c>
       <c r="H41" t="n">
-        <v>0.1318</v>
+        <v>0.031</v>
       </c>
       <c r="I41" t="n">
         <v>0.11</v>
       </c>
       <c r="J41" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -2691,7 +2691,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2745,7 +2745,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2853,7 +2853,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2911,7 +2911,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2965,7 +2965,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3019,7 +3019,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3073,7 +3073,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3082,28 +3082,28 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49" t="n">
-        <v>6.35</v>
+        <v>6.85</v>
       </c>
       <c r="E49" t="n">
-        <v>0.1046</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2641</v>
+        <v>0.2716</v>
       </c>
       <c r="G49" t="n">
-        <v>0.2119</v>
+        <v>0.1945</v>
       </c>
       <c r="H49" t="n">
-        <v>0.1372</v>
+        <v>0.1067</v>
       </c>
       <c r="I49" t="n">
-        <v>0.31</v>
+        <v>0.18</v>
       </c>
       <c r="J49" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -3115,7 +3115,7 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
@@ -3127,7 +3127,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3181,7 +3181,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3239,7 +3239,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3293,7 +3293,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3351,7 +3351,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3405,7 +3405,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3517,7 +3517,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3571,7 +3571,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3625,7 +3625,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3679,7 +3679,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3733,7 +3733,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3787,7 +3787,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3841,7 +3841,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3895,7 +3895,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3949,7 +3949,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4003,7 +4003,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4057,7 +4057,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4111,7 +4111,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4165,7 +4165,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4219,7 +4219,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4228,19 +4228,19 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
         <v>15</v>
       </c>
       <c r="E70" t="n">
-        <v>0.0158</v>
+        <v>0.0404</v>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>0.0177</v>
+        <v>0.0454</v>
       </c>
       <c r="H70" t="n">
         <v>-5.1853</v>
@@ -4261,7 +4261,7 @@
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4327,7 +4327,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4381,7 +4381,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4435,7 +4435,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4489,7 +4489,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4543,7 +4543,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4597,7 +4597,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4651,7 +4651,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4705,7 +4705,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4759,7 +4759,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4813,7 +4813,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4825,25 +4825,25 @@
         <v>8</v>
       </c>
       <c r="D81" t="n">
-        <v>1.55</v>
+        <v>2.25</v>
       </c>
       <c r="E81" t="n">
-        <v>-0.0042</v>
+        <v>0.0276</v>
       </c>
       <c r="F81" t="n">
-        <v>0.3087</v>
+        <v>0.4023</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.0136</v>
+        <v>0.0859</v>
       </c>
       <c r="H81" t="n">
-        <v>0.1315</v>
+        <v>0.2785</v>
       </c>
       <c r="I81" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="J81" t="n">
-        <v>0.41</v>
+        <v>0.42</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -4855,11 +4855,11 @@
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>⚠️ Dikkat (%7.0)</t>
+          <t>⚠️ Dikkat (%6.3)</t>
         </is>
       </c>
       <c r="R81" t="inlineStr"/>
@@ -4867,7 +4867,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4921,7 +4921,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4975,7 +4975,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5029,7 +5029,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5083,7 +5083,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5137,7 +5137,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5191,7 +5191,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5245,7 +5245,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5299,7 +5299,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5353,7 +5353,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5465,7 +5465,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5519,7 +5519,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5573,7 +5573,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5685,7 +5685,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5739,7 +5739,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5797,7 +5797,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5851,7 +5851,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5909,7 +5909,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>26.10.2026</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">

</xml_diff>